<commit_message>
feat(data): re-select 100 samples/task with weighted dialect scoring and difficulty quota
- Add select_samples_v2.py with weighted trigger scores (Negation/Template=3.0, Connective=2.0-3.0, Particle=0.5-1.0 per task)
- Filter by score>=3 OR >=2 categories instead of raw trigger count
- Add hard/medium/easy quota (30/40/30) based on category difficulty
- Track NLI trigger location (premise/hypothesis/both)
- Scan MCQA question only
- Cap dialect-signature diversity at 15 samples/signature
- Update DIALECT_LEXICON_v2.xlsx
</commit_message>
<xml_diff>
--- a/data/DIALECT_LEXICON_v2.xlsx
+++ b/data/DIALECT_LEXICON_v2.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="441">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="862" uniqueCount="442">
   <si>
     <t>#</t>
   </si>
@@ -377,6 +377,9 @@
   </si>
   <si>
     <t>cấy</t>
+  </si>
+  <si>
+    <t>cấy / kì</t>
   </si>
   <si>
     <t>bây giờ</t>
@@ -3213,7 +3216,7 @@
         <v>121</v>
       </c>
       <c r="K27" s="15" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="L27" s="15" t="s">
         <v>118</v>
@@ -3251,39 +3254,39 @@
         <v>5.0</v>
       </c>
       <c r="D28" s="15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E28" s="15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F28" s="15" t="s">
         <v>117</v>
       </c>
       <c r="G28" s="15" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H28" s="15" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I28" s="16"/>
       <c r="J28" s="16"/>
       <c r="K28" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="L28" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="M28" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="N28" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="O28" s="15" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="P28" s="15" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="Q28" s="5"/>
       <c r="R28" s="5"/>
@@ -3308,10 +3311,10 @@
         <v>6.0</v>
       </c>
       <c r="D29" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E29" s="15" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F29" s="15" t="s">
         <v>109</v>
@@ -3320,27 +3323,27 @@
         <v>40</v>
       </c>
       <c r="H29" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="I29" s="16"/>
       <c r="J29" s="16"/>
       <c r="K29" s="15" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="L29" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="M29" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="N29" s="15" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="O29" s="15" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="P29" s="15" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="Q29" s="5"/>
       <c r="R29" s="5"/>
@@ -3361,10 +3364,10 @@
     <row r="30">
       <c r="A30" s="5"/>
       <c r="B30" s="20" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C30" s="24" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="D30" s="11"/>
       <c r="E30" s="11"/>
@@ -3402,33 +3405,33 @@
         <v>1.0</v>
       </c>
       <c r="D31" s="15" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="E31" s="15" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F31" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G31" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H31" s="17" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I31" s="16"/>
       <c r="J31" s="18"/>
       <c r="K31" s="17" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="L31" s="17" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="M31" s="18"/>
       <c r="N31" s="18"/>
       <c r="O31" s="18"/>
       <c r="P31" s="17" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="Q31" s="5"/>
       <c r="R31" s="5"/>
@@ -3453,31 +3456,31 @@
         <v>2.0</v>
       </c>
       <c r="D32" s="15" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E32" s="15" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="F32" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G32" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H32" s="16"/>
       <c r="I32" s="16"/>
       <c r="J32" s="18"/>
       <c r="K32" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="L32" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M32" s="18"/>
       <c r="N32" s="18"/>
       <c r="O32" s="18"/>
       <c r="P32" s="17" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Q32" s="5"/>
       <c r="R32" s="5"/>
@@ -3502,25 +3505,25 @@
         <v>3.0</v>
       </c>
       <c r="D33" s="15" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E33" s="15" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="F33" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G33" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H33" s="18"/>
       <c r="I33" s="16"/>
       <c r="J33" s="18"/>
       <c r="K33" s="17" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="L33" s="17" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="M33" s="18"/>
       <c r="N33" s="18"/>
@@ -3549,22 +3552,22 @@
         <v>4.0</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H34" s="16"/>
       <c r="I34" s="18"/>
       <c r="J34" s="18"/>
       <c r="K34" s="17" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="L34" s="18"/>
       <c r="M34" s="18"/>
@@ -3594,31 +3597,31 @@
         <v>5.0</v>
       </c>
       <c r="D35" s="15" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="E35" s="15" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F35" s="15" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="G35" s="15" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H35" s="16"/>
       <c r="I35" s="16"/>
       <c r="J35" s="18"/>
       <c r="K35" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="L35" s="17" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="M35" s="18"/>
       <c r="N35" s="18"/>
       <c r="O35" s="18"/>
       <c r="P35" s="17" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="Q35" s="5"/>
       <c r="R35" s="5"/>
@@ -3639,10 +3642,10 @@
     <row r="36">
       <c r="A36" s="5"/>
       <c r="B36" s="23" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="C36" s="24" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="D36" s="11"/>
       <c r="E36" s="11"/>
@@ -3680,22 +3683,22 @@
         <v>1.0</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H37" s="16"/>
       <c r="I37" s="16"/>
       <c r="J37" s="18"/>
       <c r="K37" s="17" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="L37" s="18"/>
       <c r="M37" s="18"/>
@@ -3725,22 +3728,22 @@
         <v>2.0</v>
       </c>
       <c r="D38" s="15" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="E38" s="15" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F38" s="15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G38" s="15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H38" s="16"/>
       <c r="I38" s="16"/>
       <c r="J38" s="18"/>
       <c r="K38" s="17" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="L38" s="18"/>
       <c r="M38" s="18"/>
@@ -3770,16 +3773,16 @@
         <v>3.0</v>
       </c>
       <c r="D39" s="15" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E39" s="15" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F39" s="15" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="G39" s="15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H39" s="16"/>
       <c r="I39" s="16"/>
@@ -3813,22 +3816,22 @@
         <v>4.0</v>
       </c>
       <c r="D40" s="15" t="s">
+        <v>168</v>
+      </c>
+      <c r="E40" s="15" t="s">
+        <v>169</v>
+      </c>
+      <c r="F40" s="15" t="s">
         <v>167</v>
       </c>
-      <c r="E40" s="15" t="s">
-        <v>168</v>
-      </c>
-      <c r="F40" s="15" t="s">
-        <v>166</v>
-      </c>
       <c r="G40" s="15" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H40" s="16"/>
       <c r="I40" s="16"/>
       <c r="J40" s="18"/>
       <c r="K40" s="17" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="L40" s="18"/>
       <c r="M40" s="18"/>
@@ -3858,13 +3861,13 @@
         <v>5.0</v>
       </c>
       <c r="D41" s="15" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="E41" s="15" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="F41" s="15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G41" s="15" t="s">
         <v>40</v>
@@ -3901,13 +3904,13 @@
         <v>6.0</v>
       </c>
       <c r="D42" s="15" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="E42" s="15" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F42" s="15" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="G42" s="15" t="s">
         <v>40</v>
@@ -3916,14 +3919,14 @@
       <c r="I42" s="16"/>
       <c r="J42" s="18"/>
       <c r="K42" s="17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="L42" s="18"/>
       <c r="M42" s="18"/>
       <c r="N42" s="18"/>
       <c r="O42" s="18"/>
       <c r="P42" s="17" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="Q42" s="5"/>
       <c r="R42" s="5"/>
@@ -3944,10 +3947,10 @@
     <row r="43">
       <c r="A43" s="5"/>
       <c r="B43" s="20" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C43" s="24" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D43" s="11"/>
       <c r="E43" s="11"/>
@@ -3985,41 +3988,41 @@
         <v>1.0</v>
       </c>
       <c r="D44" s="15" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="E44" s="15" t="s">
+        <v>179</v>
+      </c>
+      <c r="F44" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G44" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H44" s="15" t="s">
         <v>178</v>
       </c>
-      <c r="F44" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G44" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H44" s="15" t="s">
-        <v>177</v>
-      </c>
       <c r="I44" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J44" s="18"/>
       <c r="K44" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="L44" s="15" t="s">
+        <v>184</v>
+      </c>
+      <c r="M44" s="15" t="s">
+        <v>185</v>
+      </c>
+      <c r="N44" s="15" t="s">
         <v>183</v>
       </c>
-      <c r="M44" s="15" t="s">
-        <v>184</v>
-      </c>
-      <c r="N44" s="15" t="s">
-        <v>182</v>
-      </c>
       <c r="O44" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="P44" s="15" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q44" s="5"/>
       <c r="R44" s="5"/>
@@ -4044,41 +4047,41 @@
         <v>2.0</v>
       </c>
       <c r="D45" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="E45" s="15" t="s">
+        <v>187</v>
+      </c>
+      <c r="F45" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G45" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H45" s="15" t="s">
         <v>186</v>
       </c>
-      <c r="F45" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G45" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H45" s="15" t="s">
-        <v>185</v>
-      </c>
       <c r="I45" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="J45" s="18"/>
       <c r="K45" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="L45" s="15" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="M45" s="15" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="N45" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="O45" s="15" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="P45" s="15" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="Q45" s="5"/>
       <c r="R45" s="5"/>
@@ -4103,41 +4106,41 @@
         <v>3.0</v>
       </c>
       <c r="D46" s="15" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E46" s="15" t="s">
+        <v>190</v>
+      </c>
+      <c r="F46" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G46" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H46" s="15" t="s">
         <v>189</v>
-      </c>
-      <c r="F46" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G46" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H46" s="15" t="s">
-        <v>188</v>
       </c>
       <c r="I46" s="16"/>
       <c r="J46" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="K46" s="15" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="L46" s="15" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="M46" s="15" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N46" s="15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="O46" s="15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="P46" s="15" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="Q46" s="5"/>
       <c r="R46" s="5"/>
@@ -4162,39 +4165,39 @@
         <v>4.0</v>
       </c>
       <c r="D47" s="15" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="E47" s="15" t="s">
+        <v>195</v>
+      </c>
+      <c r="F47" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G47" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H47" s="15" t="s">
         <v>194</v>
-      </c>
-      <c r="F47" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G47" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H47" s="15" t="s">
-        <v>193</v>
       </c>
       <c r="I47" s="18"/>
       <c r="J47" s="18"/>
       <c r="K47" s="15" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="L47" s="15" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="M47" s="15" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="N47" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="O47" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="P47" s="15" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="Q47" s="5"/>
       <c r="R47" s="5"/>
@@ -4219,39 +4222,39 @@
         <v>5.0</v>
       </c>
       <c r="D48" s="15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="E48" s="15" t="s">
+        <v>200</v>
+      </c>
+      <c r="F48" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G48" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H48" s="15" t="s">
         <v>199</v>
-      </c>
-      <c r="F48" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G48" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H48" s="15" t="s">
-        <v>198</v>
       </c>
       <c r="I48" s="18"/>
       <c r="J48" s="18"/>
       <c r="K48" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="L48" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="M48" s="15" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="N48" s="15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="O48" s="15" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="P48" s="15" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="Q48" s="5"/>
       <c r="R48" s="5"/>
@@ -4276,39 +4279,39 @@
         <v>6.0</v>
       </c>
       <c r="D49" s="15" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="E49" s="15" t="s">
+        <v>204</v>
+      </c>
+      <c r="F49" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G49" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H49" s="15" t="s">
         <v>203</v>
-      </c>
-      <c r="F49" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G49" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H49" s="15" t="s">
-        <v>202</v>
       </c>
       <c r="I49" s="18"/>
       <c r="J49" s="18"/>
       <c r="K49" s="15" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L49" s="15" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="M49" s="15" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="N49" s="15" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="O49" s="15" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="P49" s="15" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="Q49" s="5"/>
       <c r="R49" s="5"/>
@@ -4333,39 +4336,39 @@
         <v>7.0</v>
       </c>
       <c r="D50" s="15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="E50" s="15" t="s">
+        <v>211</v>
+      </c>
+      <c r="F50" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G50" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H50" s="15" t="s">
         <v>210</v>
-      </c>
-      <c r="F50" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G50" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H50" s="15" t="s">
-        <v>209</v>
       </c>
       <c r="I50" s="18"/>
       <c r="J50" s="18"/>
       <c r="K50" s="15" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="L50" s="15" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="M50" s="15" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="N50" s="15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="O50" s="15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="P50" s="15" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="Q50" s="5"/>
       <c r="R50" s="5"/>
@@ -4390,39 +4393,39 @@
         <v>8.0</v>
       </c>
       <c r="D51" s="15" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="E51" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="F51" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G51" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H51" s="15" t="s">
         <v>215</v>
-      </c>
-      <c r="F51" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G51" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H51" s="15" t="s">
-        <v>214</v>
       </c>
       <c r="I51" s="18"/>
       <c r="J51" s="18"/>
       <c r="K51" s="15" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="L51" s="15" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="M51" s="15" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="N51" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="O51" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="P51" s="15" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="Q51" s="5"/>
       <c r="R51" s="5"/>
@@ -4447,39 +4450,39 @@
         <v>9.0</v>
       </c>
       <c r="D52" s="15" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="E52" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="F52" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G52" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H52" s="15" t="s">
         <v>221</v>
-      </c>
-      <c r="F52" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G52" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H52" s="15" t="s">
-        <v>220</v>
       </c>
       <c r="I52" s="18"/>
       <c r="J52" s="18"/>
       <c r="K52" s="15" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="L52" s="15" t="s">
+        <v>224</v>
+      </c>
+      <c r="M52" s="15" t="s">
         <v>223</v>
       </c>
-      <c r="M52" s="15" t="s">
-        <v>222</v>
-      </c>
       <c r="N52" s="15" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="O52" s="15" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="P52" s="15" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="Q52" s="5"/>
       <c r="R52" s="5"/>
@@ -4504,39 +4507,39 @@
         <v>10.0</v>
       </c>
       <c r="D53" s="15" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="E53" s="15" t="s">
+        <v>227</v>
+      </c>
+      <c r="F53" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G53" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H53" s="15" t="s">
         <v>226</v>
-      </c>
-      <c r="F53" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G53" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H53" s="15" t="s">
-        <v>225</v>
       </c>
       <c r="I53" s="18"/>
       <c r="J53" s="18"/>
       <c r="K53" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="L53" s="15" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="M53" s="15" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="N53" s="15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="O53" s="15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="P53" s="15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="Q53" s="5"/>
       <c r="R53" s="5"/>
@@ -4561,39 +4564,39 @@
         <v>11.0</v>
       </c>
       <c r="D54" s="15" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="E54" s="15" t="s">
+        <v>232</v>
+      </c>
+      <c r="F54" s="15" t="s">
+        <v>180</v>
+      </c>
+      <c r="G54" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H54" s="15" t="s">
         <v>231</v>
-      </c>
-      <c r="F54" s="15" t="s">
-        <v>179</v>
-      </c>
-      <c r="G54" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H54" s="15" t="s">
-        <v>230</v>
       </c>
       <c r="I54" s="18"/>
       <c r="J54" s="18"/>
       <c r="K54" s="15" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="L54" s="15" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="M54" s="15" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="N54" s="15" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="O54" s="15" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="P54" s="15" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="Q54" s="5"/>
       <c r="R54" s="5"/>
@@ -4618,37 +4621,37 @@
         <v>12.0</v>
       </c>
       <c r="D55" s="15" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="E55" s="15" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="F55" s="15" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="G55" s="15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H55" s="18"/>
       <c r="I55" s="18"/>
       <c r="J55" s="18"/>
       <c r="K55" s="17" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="L55" s="17" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="M55" s="17" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="N55" s="17" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="O55" s="17" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P55" s="17" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="Q55" s="5"/>
       <c r="R55" s="5"/>
@@ -4669,10 +4672,10 @@
     <row r="56">
       <c r="A56" s="5"/>
       <c r="B56" s="23" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="C56" s="24" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="D56" s="11"/>
       <c r="E56" s="11"/>
@@ -4710,41 +4713,41 @@
         <v>1.0</v>
       </c>
       <c r="D57" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="E57" s="15" t="s">
+        <v>244</v>
+      </c>
+      <c r="F57" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="G57" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H57" s="15" t="s">
         <v>243</v>
       </c>
-      <c r="F57" s="15" t="s">
-        <v>244</v>
-      </c>
-      <c r="G57" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H57" s="15" t="s">
-        <v>242</v>
-      </c>
       <c r="I57" s="15" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="J57" s="18"/>
       <c r="K57" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="L57" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="M57" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="N57" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="O57" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="P57" s="15" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="Q57" s="5"/>
       <c r="R57" s="5"/>
@@ -4769,39 +4772,39 @@
         <v>2.0</v>
       </c>
       <c r="D58" s="15" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="E58" s="15" t="s">
+        <v>248</v>
+      </c>
+      <c r="F58" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="G58" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H58" s="15" t="s">
         <v>247</v>
-      </c>
-      <c r="F58" s="15" t="s">
-        <v>244</v>
-      </c>
-      <c r="G58" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H58" s="15" t="s">
-        <v>246</v>
       </c>
       <c r="I58" s="18"/>
       <c r="J58" s="18"/>
       <c r="K58" s="15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="L58" s="15" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="M58" s="15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="N58" s="15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="O58" s="15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="P58" s="15" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="Q58" s="5"/>
       <c r="R58" s="5"/>
@@ -4826,35 +4829,35 @@
         <v>3.0</v>
       </c>
       <c r="D59" s="15" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="E59" s="15" t="s">
+        <v>251</v>
+      </c>
+      <c r="F59" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="G59" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H59" s="15" t="s">
         <v>250</v>
-      </c>
-      <c r="F59" s="15" t="s">
-        <v>244</v>
-      </c>
-      <c r="G59" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H59" s="15" t="s">
-        <v>249</v>
       </c>
       <c r="I59" s="18"/>
       <c r="J59" s="15" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="K59" s="15" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="L59" s="15" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="M59" s="15" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="N59" s="15" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="O59" s="18"/>
       <c r="P59" s="18"/>
@@ -4881,31 +4884,31 @@
         <v>4.0</v>
       </c>
       <c r="D60" s="15" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="E60" s="15" t="s">
+        <v>254</v>
+      </c>
+      <c r="F60" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="G60" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H60" s="15" t="s">
         <v>253</v>
-      </c>
-      <c r="F60" s="15" t="s">
-        <v>244</v>
-      </c>
-      <c r="G60" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H60" s="15" t="s">
-        <v>252</v>
       </c>
       <c r="I60" s="18"/>
       <c r="J60" s="18"/>
       <c r="K60" s="15" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="L60" s="18"/>
       <c r="M60" s="15" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="N60" s="15" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="O60" s="18"/>
       <c r="P60" s="18"/>
@@ -4932,33 +4935,33 @@
         <v>5.0</v>
       </c>
       <c r="D61" s="15" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="E61" s="15" t="s">
+        <v>259</v>
+      </c>
+      <c r="F61" s="15" t="s">
+        <v>245</v>
+      </c>
+      <c r="G61" s="15" t="s">
+        <v>181</v>
+      </c>
+      <c r="H61" s="15" t="s">
         <v>258</v>
-      </c>
-      <c r="F61" s="15" t="s">
-        <v>244</v>
-      </c>
-      <c r="G61" s="15" t="s">
-        <v>180</v>
-      </c>
-      <c r="H61" s="15" t="s">
-        <v>257</v>
       </c>
       <c r="I61" s="18"/>
       <c r="J61" s="18"/>
       <c r="K61" s="15" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="L61" s="15" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="M61" s="15" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="N61" s="15" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="O61" s="18"/>
       <c r="P61" s="18"/>
@@ -4985,16 +4988,16 @@
         <v>6.0</v>
       </c>
       <c r="D62" s="15" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="E62" s="15" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="F62" s="15" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G62" s="15" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H62" s="18"/>
       <c r="I62" s="18"/>
@@ -5024,10 +5027,10 @@
     <row r="63">
       <c r="A63" s="5"/>
       <c r="B63" s="20" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
       <c r="C63" s="24" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="D63" s="11"/>
       <c r="E63" s="11"/>
@@ -5065,41 +5068,41 @@
         <v>1.0</v>
       </c>
       <c r="D64" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="E64" s="15" t="s">
+        <v>268</v>
+      </c>
+      <c r="F64" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G64" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="H64" s="15" t="s">
         <v>267</v>
       </c>
-      <c r="F64" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G64" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="H64" s="15" t="s">
-        <v>266</v>
-      </c>
       <c r="I64" s="15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="J64" s="18"/>
       <c r="K64" s="15" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
       <c r="L64" s="15" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="M64" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="N64" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="O64" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="P64" s="15" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="Q64" s="5"/>
       <c r="R64" s="5"/>
@@ -5124,39 +5127,39 @@
         <v>2.0</v>
       </c>
       <c r="D65" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="E65" s="15" t="s">
+        <v>274</v>
+      </c>
+      <c r="F65" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G65" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="H65" s="15" t="s">
         <v>273</v>
-      </c>
-      <c r="F65" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G65" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="H65" s="15" t="s">
-        <v>272</v>
       </c>
       <c r="I65" s="18"/>
       <c r="J65" s="18"/>
       <c r="K65" s="15" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="L65" s="15" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="M65" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="N65" s="15" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="O65" s="15" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="P65" s="15" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="Q65" s="5"/>
       <c r="R65" s="5"/>
@@ -5181,22 +5184,22 @@
         <v>3.0</v>
       </c>
       <c r="D66" s="15" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="E66" s="15" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="F66" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G66" s="15" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H66" s="18"/>
       <c r="I66" s="18"/>
       <c r="J66" s="18"/>
       <c r="K66" s="17" t="s">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="L66" s="18"/>
       <c r="M66" s="18"/>
@@ -5226,41 +5229,41 @@
         <v>4.0</v>
       </c>
       <c r="D67" s="15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="E67" s="15" t="s">
+        <v>281</v>
+      </c>
+      <c r="F67" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G67" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="H67" s="15" t="s">
         <v>280</v>
       </c>
-      <c r="F67" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G67" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="H67" s="15" t="s">
-        <v>279</v>
-      </c>
       <c r="I67" s="15" t="s">
-        <v>281</v>
+        <v>282</v>
       </c>
       <c r="J67" s="18"/>
       <c r="K67" s="15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="L67" s="15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="M67" s="15" t="s">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="N67" s="15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="O67" s="15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="P67" s="15" t="s">
-        <v>282</v>
+        <v>283</v>
       </c>
       <c r="Q67" s="5"/>
       <c r="R67" s="5"/>
@@ -5285,16 +5288,16 @@
         <v>5.0</v>
       </c>
       <c r="D68" s="15" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="E68" s="15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
       <c r="F68" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G68" s="15" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="H68" s="18"/>
       <c r="I68" s="18"/>
@@ -5328,26 +5331,26 @@
         <v>6.0</v>
       </c>
       <c r="D69" s="15" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
       <c r="E69" s="15" t="s">
+        <v>287</v>
+      </c>
+      <c r="F69" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G69" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H69" s="15" t="s">
         <v>286</v>
-      </c>
-      <c r="F69" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G69" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H69" s="15" t="s">
-        <v>285</v>
       </c>
       <c r="I69" s="18"/>
       <c r="J69" s="15" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K69" s="15" t="s">
-        <v>289</v>
+        <v>290</v>
       </c>
       <c r="L69" s="18"/>
       <c r="M69" s="18"/>
@@ -5377,16 +5380,16 @@
         <v>7.0</v>
       </c>
       <c r="D70" s="15" t="s">
-        <v>290</v>
+        <v>291</v>
       </c>
       <c r="E70" s="15" t="s">
-        <v>291</v>
+        <v>292</v>
       </c>
       <c r="F70" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G70" s="15" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H70" s="18"/>
       <c r="I70" s="18"/>
@@ -5420,29 +5423,29 @@
         <v>8.0</v>
       </c>
       <c r="D71" s="15" t="s">
-        <v>292</v>
+        <v>293</v>
       </c>
       <c r="E71" s="15" t="s">
+        <v>294</v>
+      </c>
+      <c r="F71" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G71" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H71" s="15" t="s">
         <v>293</v>
-      </c>
-      <c r="F71" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G71" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H71" s="15" t="s">
-        <v>292</v>
       </c>
       <c r="I71" s="18"/>
       <c r="J71" s="15" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="K71" s="15" t="s">
+        <v>296</v>
+      </c>
+      <c r="L71" s="15" t="s">
         <v>295</v>
-      </c>
-      <c r="L71" s="15" t="s">
-        <v>294</v>
       </c>
       <c r="M71" s="18"/>
       <c r="N71" s="18"/>
@@ -5471,39 +5474,39 @@
         <v>9.0</v>
       </c>
       <c r="D72" s="15" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E72" s="15" t="s">
+        <v>298</v>
+      </c>
+      <c r="F72" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G72" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H72" s="15" t="s">
         <v>297</v>
-      </c>
-      <c r="F72" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G72" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H72" s="15" t="s">
-        <v>296</v>
       </c>
       <c r="I72" s="18"/>
       <c r="J72" s="18"/>
       <c r="K72" s="15" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="L72" s="15" t="s">
-        <v>299</v>
+        <v>300</v>
       </c>
       <c r="M72" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="N72" s="15" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="O72" s="15" t="s">
+        <v>302</v>
+      </c>
+      <c r="P72" s="15" t="s">
         <v>301</v>
-      </c>
-      <c r="P72" s="15" t="s">
-        <v>300</v>
       </c>
       <c r="Q72" s="5"/>
       <c r="R72" s="5"/>
@@ -5528,39 +5531,39 @@
         <v>10.0</v>
       </c>
       <c r="D73" s="15" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="E73" s="15" t="s">
+        <v>304</v>
+      </c>
+      <c r="F73" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G73" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="H73" s="15" t="s">
         <v>303</v>
-      </c>
-      <c r="F73" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G73" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="H73" s="15" t="s">
-        <v>302</v>
       </c>
       <c r="I73" s="18"/>
       <c r="J73" s="18"/>
       <c r="K73" s="15" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="L73" s="15" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="M73" s="15" t="s">
-        <v>302</v>
+        <v>303</v>
       </c>
       <c r="N73" s="15" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="O73" s="15" t="s">
+        <v>307</v>
+      </c>
+      <c r="P73" s="15" t="s">
         <v>306</v>
-      </c>
-      <c r="P73" s="15" t="s">
-        <v>305</v>
       </c>
       <c r="Q73" s="5"/>
       <c r="R73" s="5"/>
@@ -5585,39 +5588,39 @@
         <v>11.0</v>
       </c>
       <c r="D74" s="15" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="E74" s="15" t="s">
+        <v>309</v>
+      </c>
+      <c r="F74" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G74" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="H74" s="15" t="s">
         <v>308</v>
-      </c>
-      <c r="F74" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G74" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="H74" s="15" t="s">
-        <v>307</v>
       </c>
       <c r="I74" s="18"/>
       <c r="J74" s="18"/>
       <c r="K74" s="15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="L74" s="15" t="s">
-        <v>309</v>
+        <v>310</v>
       </c>
       <c r="M74" s="15" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="N74" s="15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="O74" s="15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="P74" s="15" t="s">
-        <v>310</v>
+        <v>311</v>
       </c>
       <c r="Q74" s="5"/>
       <c r="R74" s="5"/>
@@ -5642,31 +5645,31 @@
         <v>12.0</v>
       </c>
       <c r="D75" s="15" t="s">
-        <v>311</v>
+        <v>312</v>
       </c>
       <c r="E75" s="15" t="s">
+        <v>313</v>
+      </c>
+      <c r="F75" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G75" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H75" s="15" t="s">
         <v>312</v>
-      </c>
-      <c r="F75" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G75" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H75" s="15" t="s">
-        <v>311</v>
       </c>
       <c r="I75" s="18"/>
       <c r="J75" s="18"/>
       <c r="K75" s="15" t="s">
-        <v>313</v>
+        <v>314</v>
       </c>
       <c r="L75" s="18"/>
       <c r="M75" s="15" t="s">
-        <v>314</v>
+        <v>315</v>
       </c>
       <c r="N75" s="15" t="s">
-        <v>315</v>
+        <v>316</v>
       </c>
       <c r="O75" s="18"/>
       <c r="P75" s="18"/>
@@ -5693,25 +5696,25 @@
         <v>13.0</v>
       </c>
       <c r="D76" s="15" t="s">
-        <v>316</v>
+        <v>317</v>
       </c>
       <c r="E76" s="15" t="s">
+        <v>318</v>
+      </c>
+      <c r="F76" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G76" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="H76" s="15" t="s">
         <v>317</v>
-      </c>
-      <c r="F76" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G76" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="H76" s="15" t="s">
-        <v>316</v>
       </c>
       <c r="I76" s="18"/>
       <c r="J76" s="18"/>
       <c r="K76" s="18"/>
       <c r="L76" s="15" t="s">
-        <v>318</v>
+        <v>319</v>
       </c>
       <c r="M76" s="18"/>
       <c r="N76" s="18"/>
@@ -5740,24 +5743,24 @@
         <v>14.0</v>
       </c>
       <c r="D77" s="15" t="s">
-        <v>319</v>
+        <v>320</v>
       </c>
       <c r="E77" s="15" t="s">
+        <v>321</v>
+      </c>
+      <c r="F77" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G77" s="15" t="s">
+        <v>270</v>
+      </c>
+      <c r="H77" s="15" t="s">
         <v>320</v>
-      </c>
-      <c r="F77" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G77" s="15" t="s">
-        <v>269</v>
-      </c>
-      <c r="H77" s="15" t="s">
-        <v>319</v>
       </c>
       <c r="I77" s="18"/>
       <c r="J77" s="18"/>
       <c r="K77" s="15" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="L77" s="18"/>
       <c r="M77" s="18"/>
@@ -5787,33 +5790,33 @@
         <v>15.0</v>
       </c>
       <c r="D78" s="15" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="E78" s="15" t="s">
+        <v>324</v>
+      </c>
+      <c r="F78" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G78" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H78" s="15" t="s">
         <v>323</v>
-      </c>
-      <c r="F78" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G78" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H78" s="15" t="s">
-        <v>322</v>
       </c>
       <c r="I78" s="18"/>
       <c r="J78" s="15" t="s">
-        <v>324</v>
+        <v>325</v>
       </c>
       <c r="K78" s="15" t="s">
-        <v>325</v>
+        <v>326</v>
       </c>
       <c r="L78" s="18"/>
       <c r="M78" s="15" t="s">
-        <v>326</v>
+        <v>327</v>
       </c>
       <c r="N78" s="15" t="s">
-        <v>327</v>
+        <v>328</v>
       </c>
       <c r="O78" s="18"/>
       <c r="P78" s="18"/>
@@ -5840,37 +5843,37 @@
         <v>16.0</v>
       </c>
       <c r="D79" s="15" t="s">
-        <v>328</v>
+        <v>329</v>
       </c>
       <c r="E79" s="15" t="s">
+        <v>330</v>
+      </c>
+      <c r="F79" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G79" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H79" s="15" t="s">
         <v>329</v>
       </c>
-      <c r="F79" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G79" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H79" s="15" t="s">
-        <v>328</v>
-      </c>
       <c r="I79" s="15" t="s">
-        <v>330</v>
+        <v>331</v>
       </c>
       <c r="J79" s="15" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="K79" s="15" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="L79" s="15" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="M79" s="15" t="s">
-        <v>333</v>
+        <v>334</v>
       </c>
       <c r="N79" s="15" t="s">
-        <v>334</v>
+        <v>335</v>
       </c>
       <c r="O79" s="18"/>
       <c r="P79" s="18"/>
@@ -5897,33 +5900,33 @@
         <v>17.0</v>
       </c>
       <c r="D80" s="15" t="s">
-        <v>335</v>
+        <v>336</v>
       </c>
       <c r="E80" s="15" t="s">
+        <v>337</v>
+      </c>
+      <c r="F80" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G80" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H80" s="15" t="s">
         <v>336</v>
-      </c>
-      <c r="F80" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G80" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H80" s="15" t="s">
-        <v>335</v>
       </c>
       <c r="I80" s="18"/>
       <c r="J80" s="15" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="K80" s="15" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="L80" s="15" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="M80" s="18"/>
       <c r="N80" s="15" t="s">
-        <v>340</v>
+        <v>341</v>
       </c>
       <c r="O80" s="18"/>
       <c r="P80" s="18"/>
@@ -5950,31 +5953,31 @@
         <v>18.0</v>
       </c>
       <c r="D81" s="15" t="s">
-        <v>341</v>
+        <v>342</v>
       </c>
       <c r="E81" s="15" t="s">
+        <v>343</v>
+      </c>
+      <c r="F81" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G81" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H81" s="15" t="s">
         <v>342</v>
-      </c>
-      <c r="F81" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G81" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H81" s="15" t="s">
-        <v>341</v>
       </c>
       <c r="I81" s="18"/>
       <c r="J81" s="18"/>
       <c r="K81" s="15" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="L81" s="18"/>
       <c r="M81" s="15" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="N81" s="15" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="O81" s="18"/>
       <c r="P81" s="18"/>
@@ -6001,39 +6004,39 @@
         <v>19.0</v>
       </c>
       <c r="D82" s="15" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="E82" s="15" t="s">
+        <v>348</v>
+      </c>
+      <c r="F82" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G82" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H82" s="15" t="s">
         <v>347</v>
-      </c>
-      <c r="F82" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G82" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H82" s="15" t="s">
-        <v>346</v>
       </c>
       <c r="I82" s="18"/>
       <c r="J82" s="15" t="s">
-        <v>348</v>
+        <v>349</v>
       </c>
       <c r="K82" s="15" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="L82" s="15" t="s">
+        <v>351</v>
+      </c>
+      <c r="M82" s="15" t="s">
         <v>350</v>
       </c>
-      <c r="M82" s="15" t="s">
-        <v>349</v>
-      </c>
       <c r="N82" s="15" t="s">
-        <v>349</v>
+        <v>350</v>
       </c>
       <c r="O82" s="18"/>
       <c r="P82" s="15" t="s">
-        <v>351</v>
+        <v>352</v>
       </c>
       <c r="Q82" s="5"/>
       <c r="R82" s="5"/>
@@ -6058,29 +6061,29 @@
         <v>20.0</v>
       </c>
       <c r="D83" s="15" t="s">
-        <v>352</v>
+        <v>353</v>
       </c>
       <c r="E83" s="15" t="s">
-        <v>353</v>
+        <v>354</v>
       </c>
       <c r="F83" s="15" t="s">
-        <v>268</v>
+        <v>269</v>
       </c>
       <c r="G83" s="15" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="H83" s="15" t="s">
-        <v>354</v>
+        <v>355</v>
       </c>
       <c r="I83" s="18"/>
       <c r="J83" s="17" t="s">
-        <v>288</v>
+        <v>289</v>
       </c>
       <c r="K83" s="15" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="L83" s="15" t="s">
-        <v>355</v>
+        <v>356</v>
       </c>
       <c r="M83" s="18"/>
       <c r="N83" s="18"/>
@@ -6109,36 +6112,36 @@
         <v>21.0</v>
       </c>
       <c r="D84" s="15" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="E84" s="15" t="s">
+        <v>358</v>
+      </c>
+      <c r="F84" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G84" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="H84" s="15" t="s">
         <v>357</v>
-      </c>
-      <c r="F84" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G84" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H84" s="15" t="s">
-        <v>356</v>
       </c>
       <c r="I84" s="18"/>
       <c r="J84" s="18"/>
       <c r="K84" s="15" t="s">
-        <v>359</v>
+        <v>360</v>
       </c>
       <c r="L84" s="15" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="M84" s="15" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="N84" s="15" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="O84" s="15" t="s">
-        <v>356</v>
+        <v>357</v>
       </c>
       <c r="P84" s="18"/>
       <c r="Q84" s="5"/>
@@ -6164,39 +6167,39 @@
         <v>22.0</v>
       </c>
       <c r="D85" s="15" t="s">
-        <v>360</v>
+        <v>361</v>
       </c>
       <c r="E85" s="15" t="s">
+        <v>362</v>
+      </c>
+      <c r="F85" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G85" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="H85" s="15" t="s">
         <v>361</v>
-      </c>
-      <c r="F85" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G85" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H85" s="15" t="s">
-        <v>360</v>
       </c>
       <c r="I85" s="18"/>
       <c r="J85" s="18"/>
       <c r="K85" s="15" t="s">
-        <v>362</v>
+        <v>363</v>
       </c>
       <c r="L85" s="15" t="s">
-        <v>363</v>
+        <v>364</v>
       </c>
       <c r="M85" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="N85" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="O85" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="P85" s="15" t="s">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="Q85" s="5"/>
       <c r="R85" s="5"/>
@@ -6221,26 +6224,26 @@
         <v>23.0</v>
       </c>
       <c r="D86" s="15" t="s">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="E86" s="15" t="s">
+        <v>367</v>
+      </c>
+      <c r="F86" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G86" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="H86" s="15" t="s">
         <v>366</v>
-      </c>
-      <c r="F86" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G86" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H86" s="15" t="s">
-        <v>365</v>
       </c>
       <c r="I86" s="18"/>
       <c r="J86" s="15" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="K86" s="15" t="s">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="L86" s="18"/>
       <c r="M86" s="18"/>
@@ -6270,26 +6273,26 @@
         <v>24.0</v>
       </c>
       <c r="D87" s="15" t="s">
-        <v>368</v>
+        <v>369</v>
       </c>
       <c r="E87" s="15" t="s">
+        <v>370</v>
+      </c>
+      <c r="F87" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G87" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="H87" s="15" t="s">
         <v>369</v>
-      </c>
-      <c r="F87" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G87" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H87" s="15" t="s">
-        <v>368</v>
       </c>
       <c r="I87" s="18"/>
       <c r="J87" s="15" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="K87" s="15" t="s">
-        <v>370</v>
+        <v>371</v>
       </c>
       <c r="L87" s="18"/>
       <c r="M87" s="18"/>
@@ -6319,33 +6322,33 @@
         <v>25.0</v>
       </c>
       <c r="D88" s="15" t="s">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="E88" s="15" t="s">
+        <v>373</v>
+      </c>
+      <c r="F88" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G88" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H88" s="15" t="s">
         <v>372</v>
-      </c>
-      <c r="F88" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G88" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H88" s="15" t="s">
-        <v>371</v>
       </c>
       <c r="I88" s="18"/>
       <c r="J88" s="15" t="s">
-        <v>373</v>
+        <v>374</v>
       </c>
       <c r="K88" s="15" t="s">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="L88" s="18"/>
       <c r="M88" s="15" t="s">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="N88" s="15" t="s">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="O88" s="18"/>
       <c r="P88" s="18"/>
@@ -6372,29 +6375,29 @@
         <v>26.0</v>
       </c>
       <c r="D89" s="15" t="s">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="E89" s="15" t="s">
+        <v>379</v>
+      </c>
+      <c r="F89" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G89" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="H89" s="15" t="s">
         <v>378</v>
-      </c>
-      <c r="F89" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G89" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H89" s="15" t="s">
-        <v>377</v>
       </c>
       <c r="I89" s="18"/>
       <c r="J89" s="18"/>
       <c r="K89" s="15" t="s">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="L89" s="18"/>
       <c r="M89" s="18"/>
       <c r="N89" s="15" t="s">
-        <v>380</v>
+        <v>381</v>
       </c>
       <c r="O89" s="18"/>
       <c r="P89" s="18"/>
@@ -6421,29 +6424,29 @@
         <v>27.0</v>
       </c>
       <c r="D90" s="15" t="s">
-        <v>381</v>
+        <v>382</v>
       </c>
       <c r="E90" s="15" t="s">
+        <v>383</v>
+      </c>
+      <c r="F90" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G90" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="H90" s="15" t="s">
         <v>382</v>
-      </c>
-      <c r="F90" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G90" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H90" s="15" t="s">
-        <v>381</v>
       </c>
       <c r="I90" s="18"/>
       <c r="J90" s="18"/>
       <c r="K90" s="15" t="s">
-        <v>383</v>
+        <v>384</v>
       </c>
       <c r="L90" s="18"/>
       <c r="M90" s="18"/>
       <c r="N90" s="15" t="s">
-        <v>384</v>
+        <v>385</v>
       </c>
       <c r="O90" s="18"/>
       <c r="P90" s="18"/>
@@ -6470,24 +6473,24 @@
         <v>28.0</v>
       </c>
       <c r="D91" s="15" t="s">
-        <v>385</v>
+        <v>386</v>
       </c>
       <c r="E91" s="15" t="s">
+        <v>387</v>
+      </c>
+      <c r="F91" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G91" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="H91" s="15" t="s">
         <v>386</v>
-      </c>
-      <c r="F91" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G91" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H91" s="15" t="s">
-        <v>385</v>
       </c>
       <c r="I91" s="18"/>
       <c r="J91" s="18"/>
       <c r="K91" s="15" t="s">
-        <v>387</v>
+        <v>388</v>
       </c>
       <c r="L91" s="18"/>
       <c r="M91" s="18"/>
@@ -6517,33 +6520,33 @@
         <v>29.0</v>
       </c>
       <c r="D92" s="15" t="s">
-        <v>388</v>
+        <v>389</v>
       </c>
       <c r="E92" s="15" t="s">
+        <v>390</v>
+      </c>
+      <c r="F92" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G92" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H92" s="15" t="s">
         <v>389</v>
       </c>
-      <c r="F92" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G92" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H92" s="15" t="s">
-        <v>388</v>
-      </c>
       <c r="I92" s="15" t="s">
-        <v>390</v>
+        <v>391</v>
       </c>
       <c r="J92" s="15" t="s">
-        <v>391</v>
+        <v>392</v>
       </c>
       <c r="K92" s="15" t="s">
-        <v>392</v>
+        <v>393</v>
       </c>
       <c r="L92" s="18"/>
       <c r="M92" s="18"/>
       <c r="N92" s="15" t="s">
-        <v>393</v>
+        <v>394</v>
       </c>
       <c r="O92" s="18"/>
       <c r="P92" s="18"/>
@@ -6570,24 +6573,24 @@
         <v>30.0</v>
       </c>
       <c r="D93" s="15" t="s">
-        <v>394</v>
+        <v>395</v>
       </c>
       <c r="E93" s="15" t="s">
+        <v>396</v>
+      </c>
+      <c r="F93" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G93" s="15" t="s">
+        <v>288</v>
+      </c>
+      <c r="H93" s="15" t="s">
         <v>395</v>
-      </c>
-      <c r="F93" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G93" s="15" t="s">
-        <v>287</v>
-      </c>
-      <c r="H93" s="15" t="s">
-        <v>394</v>
       </c>
       <c r="I93" s="18"/>
       <c r="J93" s="18"/>
       <c r="K93" s="15" t="s">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="L93" s="18"/>
       <c r="M93" s="18"/>
@@ -6617,29 +6620,29 @@
         <v>31.0</v>
       </c>
       <c r="D94" s="15" t="s">
-        <v>397</v>
+        <v>398</v>
       </c>
       <c r="E94" s="15" t="s">
+        <v>399</v>
+      </c>
+      <c r="F94" s="15" t="s">
+        <v>269</v>
+      </c>
+      <c r="G94" s="15" t="s">
+        <v>359</v>
+      </c>
+      <c r="H94" s="15" t="s">
         <v>398</v>
       </c>
-      <c r="F94" s="15" t="s">
-        <v>268</v>
-      </c>
-      <c r="G94" s="15" t="s">
-        <v>358</v>
-      </c>
-      <c r="H94" s="15" t="s">
-        <v>397</v>
-      </c>
       <c r="I94" s="15" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="J94" s="18"/>
       <c r="K94" s="15" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="L94" s="15" t="s">
-        <v>399</v>
+        <v>400</v>
       </c>
       <c r="M94" s="18"/>
       <c r="N94" s="18"/>
@@ -6664,10 +6667,10 @@
     <row r="95">
       <c r="A95" s="5"/>
       <c r="B95" s="23" t="s">
-        <v>400</v>
+        <v>401</v>
       </c>
       <c r="C95" s="24" t="s">
-        <v>401</v>
+        <v>402</v>
       </c>
       <c r="D95" s="11"/>
       <c r="E95" s="11"/>
@@ -6705,29 +6708,29 @@
         <v>1.0</v>
       </c>
       <c r="D96" s="15" t="s">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="E96" s="15" t="s">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="F96" s="15" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G96" s="15" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="H96" s="18"/>
       <c r="I96" s="17" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="J96" s="17" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="K96" s="17" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="L96" s="17" t="s">
-        <v>406</v>
+        <v>407</v>
       </c>
       <c r="M96" s="18"/>
       <c r="N96" s="18"/>
@@ -6756,29 +6759,29 @@
         <v>2.0</v>
       </c>
       <c r="D97" s="15" t="s">
-        <v>407</v>
+        <v>408</v>
       </c>
       <c r="E97" s="15" t="s">
-        <v>408</v>
+        <v>409</v>
       </c>
       <c r="F97" s="15" t="s">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="G97" s="15" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="H97" s="17" t="s">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="I97" s="18"/>
       <c r="J97" s="17" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="K97" s="17" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="L97" s="17" t="s">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="M97" s="18"/>
       <c r="N97" s="18"/>
@@ -6807,27 +6810,27 @@
         <v>3.0</v>
       </c>
       <c r="D98" s="15" t="s">
-        <v>411</v>
+        <v>412</v>
       </c>
       <c r="E98" s="15" t="s">
+        <v>413</v>
+      </c>
+      <c r="F98" s="15" t="s">
+        <v>405</v>
+      </c>
+      <c r="G98" s="15" t="s">
+        <v>406</v>
+      </c>
+      <c r="H98" s="17" t="s">
         <v>412</v>
-      </c>
-      <c r="F98" s="15" t="s">
-        <v>404</v>
-      </c>
-      <c r="G98" s="15" t="s">
-        <v>405</v>
-      </c>
-      <c r="H98" s="17" t="s">
-        <v>411</v>
       </c>
       <c r="I98" s="18"/>
       <c r="J98" s="18"/>
       <c r="K98" s="17" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="L98" s="17" t="s">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="M98" s="18"/>
       <c r="N98" s="18"/>
@@ -6856,19 +6859,19 @@
         <v>4.0</v>
       </c>
       <c r="D99" s="15" t="s">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="E99" s="15" t="s">
-        <v>415</v>
+        <v>416</v>
       </c>
       <c r="F99" s="15" t="s">
-        <v>416</v>
+        <v>417</v>
       </c>
       <c r="G99" s="15" t="s">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="H99" s="17" t="s">
-        <v>417</v>
+        <v>418</v>
       </c>
       <c r="I99" s="18"/>
       <c r="J99" s="18"/>
@@ -6901,39 +6904,39 @@
         <v>5.0</v>
       </c>
       <c r="D100" s="15" t="s">
-        <v>418</v>
+        <v>419</v>
       </c>
       <c r="E100" s="15" t="s">
+        <v>420</v>
+      </c>
+      <c r="F100" s="15" t="s">
+        <v>417</v>
+      </c>
+      <c r="G100" s="15" t="s">
+        <v>406</v>
+      </c>
+      <c r="H100" s="15" t="s">
         <v>419</v>
-      </c>
-      <c r="F100" s="15" t="s">
-        <v>416</v>
-      </c>
-      <c r="G100" s="15" t="s">
-        <v>405</v>
-      </c>
-      <c r="H100" s="15" t="s">
-        <v>418</v>
       </c>
       <c r="I100" s="18"/>
       <c r="J100" s="18"/>
       <c r="K100" s="15" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="L100" s="15" t="s">
-        <v>420</v>
+        <v>421</v>
       </c>
       <c r="M100" s="15" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="N100" s="15" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="O100" s="15" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="P100" s="15" t="s">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="Q100" s="5"/>
       <c r="R100" s="5"/>
@@ -6958,38 +6961,38 @@
         <v>6.0</v>
       </c>
       <c r="D101" s="15" t="s">
-        <v>422</v>
+        <v>423</v>
       </c>
       <c r="E101" s="15" t="s">
+        <v>424</v>
+      </c>
+      <c r="F101" s="15" t="s">
+        <v>417</v>
+      </c>
+      <c r="G101" s="15" t="s">
+        <v>406</v>
+      </c>
+      <c r="H101" s="15" t="s">
         <v>423</v>
       </c>
-      <c r="F101" s="15" t="s">
-        <v>416</v>
-      </c>
-      <c r="G101" s="15" t="s">
-        <v>405</v>
-      </c>
-      <c r="H101" s="15" t="s">
-        <v>422</v>
-      </c>
       <c r="I101" s="15" t="s">
-        <v>424</v>
+        <v>425</v>
       </c>
       <c r="J101" s="18"/>
       <c r="K101" s="15" t="s">
-        <v>425</v>
+        <v>426</v>
       </c>
       <c r="L101" s="15" t="s">
-        <v>426</v>
+        <v>427</v>
       </c>
       <c r="M101" s="15" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="N101" s="15" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="O101" s="15" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="P101" s="18"/>
       <c r="Q101" s="5"/>
@@ -7015,39 +7018,39 @@
         <v>7.0</v>
       </c>
       <c r="D102" s="15" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="E102" s="15" t="s">
+        <v>432</v>
+      </c>
+      <c r="F102" s="15" t="s">
+        <v>417</v>
+      </c>
+      <c r="G102" s="15" t="s">
+        <v>406</v>
+      </c>
+      <c r="H102" s="15" t="s">
         <v>431</v>
-      </c>
-      <c r="F102" s="15" t="s">
-        <v>416</v>
-      </c>
-      <c r="G102" s="15" t="s">
-        <v>405</v>
-      </c>
-      <c r="H102" s="15" t="s">
-        <v>430</v>
       </c>
       <c r="I102" s="18"/>
       <c r="J102" s="18"/>
       <c r="K102" s="15" t="s">
-        <v>432</v>
+        <v>433</v>
       </c>
       <c r="L102" s="15" t="s">
-        <v>433</v>
+        <v>434</v>
       </c>
       <c r="M102" s="15" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="N102" s="15" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="O102" s="15" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="P102" s="15" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
       <c r="Q102" s="5"/>
       <c r="R102" s="5"/>
@@ -7072,39 +7075,39 @@
         <v>8.0</v>
       </c>
       <c r="D103" s="15" t="s">
-        <v>435</v>
+        <v>436</v>
       </c>
       <c r="E103" s="15" t="s">
+        <v>437</v>
+      </c>
+      <c r="F103" s="15" t="s">
+        <v>417</v>
+      </c>
+      <c r="G103" s="15" t="s">
+        <v>406</v>
+      </c>
+      <c r="H103" s="15" t="s">
         <v>436</v>
-      </c>
-      <c r="F103" s="15" t="s">
-        <v>416</v>
-      </c>
-      <c r="G103" s="15" t="s">
-        <v>405</v>
-      </c>
-      <c r="H103" s="15" t="s">
-        <v>435</v>
       </c>
       <c r="I103" s="18"/>
       <c r="J103" s="18"/>
       <c r="K103" s="15" t="s">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="L103" s="15" t="s">
-        <v>438</v>
+        <v>439</v>
       </c>
       <c r="M103" s="15" t="s">
-        <v>439</v>
+        <v>440</v>
       </c>
       <c r="N103" s="15" t="s">
+        <v>441</v>
+      </c>
+      <c r="O103" s="15" t="s">
         <v>440</v>
       </c>
-      <c r="O103" s="15" t="s">
-        <v>439</v>
-      </c>
       <c r="P103" s="15" t="s">
-        <v>440</v>
+        <v>441</v>
       </c>
       <c r="Q103" s="5"/>
       <c r="R103" s="5"/>
@@ -36296,24 +36299,24 @@
     </row>
   </sheetData>
   <mergeCells count="18">
-    <mergeCell ref="B3:B11"/>
-    <mergeCell ref="C3:P3"/>
-    <mergeCell ref="C12:P12"/>
-    <mergeCell ref="B12:B22"/>
-    <mergeCell ref="C23:P23"/>
-    <mergeCell ref="B23:B29"/>
     <mergeCell ref="B30:B35"/>
+    <mergeCell ref="B36:B42"/>
+    <mergeCell ref="B43:B55"/>
     <mergeCell ref="B56:B62"/>
     <mergeCell ref="B63:B94"/>
     <mergeCell ref="B95:B103"/>
-    <mergeCell ref="C30:P30"/>
     <mergeCell ref="C36:P36"/>
-    <mergeCell ref="B36:B42"/>
     <mergeCell ref="C43:P43"/>
-    <mergeCell ref="B43:B55"/>
     <mergeCell ref="C56:P56"/>
     <mergeCell ref="C63:P63"/>
     <mergeCell ref="C95:P95"/>
+    <mergeCell ref="B3:B11"/>
+    <mergeCell ref="C3:P3"/>
+    <mergeCell ref="B12:B22"/>
+    <mergeCell ref="C12:P12"/>
+    <mergeCell ref="B23:B29"/>
+    <mergeCell ref="C23:P23"/>
+    <mergeCell ref="C30:P30"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>